<commit_message>
Update MediBot: Implement ReAct agent with natural English responses, JSON-to-text conversion, improved prompt templates, and session memory
</commit_message>
<xml_diff>
--- a/Evaluation Rubrics - Medibot.xlsx
+++ b/Evaluation Rubrics - Medibot.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debo/Documents/IK/CapstoneProjects/MediBot/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debo/Documents/Projects/MLAI/CapstoneProjects/mlai-capstone-medibot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D19FC8E2-3F7D-9A48-A0F5-61907960B50A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A292E21D-BF88-F04F-B37D-F9BBC82BBCB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,20 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="ProblemStatement" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -293,6 +306,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>based on symptom inputs.</t>
@@ -317,6 +331,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>to guide users on urgency.</t>
@@ -344,6 +359,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>and self-care recommendations.</t>
@@ -812,6 +828,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>to let the AI </t>
@@ -841,6 +858,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>the right agent.</t>
@@ -875,6 +893,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>to track symptom progression over multiple interactions.</t>
@@ -909,6 +928,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>for efficient </t>
@@ -1096,6 +1116,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>(symptom checking, severity assessment, disease descriptions, precautions).</t>
@@ -1130,6 +1151,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>for autonomous decision-making.</t>
@@ -1164,6 +1186,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>and improvements needed.</t>
@@ -1201,6 +1224,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>(symptom-disease mapping, severity scores, medical guidelines).</t>
@@ -1253,6 +1277,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>for better understanding.</t>
@@ -1287,6 +1312,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>for retrieval.</t>
@@ -1321,6 +1347,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>for efficient symptom retrieval.</t>
@@ -1383,6 +1410,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>– Predicts illnesses based on symptoms.</t>
@@ -1417,6 +1445,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>– Assesses urgency.</t>
@@ -1451,6 +1480,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>– Provides explanations.</t>
@@ -1485,6 +1515,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>– Suggests preventive measures.</t>
@@ -1529,6 +1560,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>to register agents.</t>
@@ -1591,6 +1623,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>to dynamically select agents.</t>
@@ -1625,6 +1658,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>and route them correctly.</t>
@@ -1771,6 +1805,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>(deploy on Hugging Face Spaces or AWS).</t>
@@ -1805,6 +1840,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>to refine model accuracy.</t>
@@ -1867,6 +1903,7 @@
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>for AI-driven medical assistance.</t>
@@ -2008,18 +2045,21 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -30448,458 +30488,459 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EE0A16F-2ADA-F34E-AC9C-AC7F25E49DB5}">
-  <dimension ref="A1:A117"/>
+  <dimension ref="B1:B117"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="30" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="2:2" ht="30" x14ac:dyDescent="0.3">
+      <c r="B1" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="2:2" ht="18" x14ac:dyDescent="0.2">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B4" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B6" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B8" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B10" s="7" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A11" s="8" t="s">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B11" s="8" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A12" s="8" t="s">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B12" s="8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A13" s="8" t="s">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B13" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A14" s="8" t="s">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B14" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B16" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="6" t="s">
+    <row r="19" spans="2:2" ht="18" x14ac:dyDescent="0.2">
+      <c r="B19" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B20" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A21" s="7" t="s">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B21" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A22" s="7" t="s">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B22" s="7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A23" s="7" t="s">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B23" s="7" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A25" s="7" t="s">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B25" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A27" s="7" t="s">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B27" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A28" s="8" t="s">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B28" s="8" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A29" s="8" t="s">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B29" s="8" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A30" s="8" t="s">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B30" s="8" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A31" s="8" t="s">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B31" s="8" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A33" s="7" t="s">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B33" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A36" s="6" t="s">
+    <row r="36" spans="2:2" ht="18" x14ac:dyDescent="0.2">
+      <c r="B36" s="6" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A37" s="7" t="s">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B37" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A38" s="7" t="s">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B38" s="7" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A39" s="8" t="s">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B39" s="8" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A40" s="8" t="s">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B40" s="8" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A41" s="8" t="s">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B41" s="8" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A42" s="8" t="s">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B42" s="8" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A43" s="7" t="s">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B43" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A44" s="7" t="s">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B44" s="7" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A45" s="7" t="s">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B45" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A46" s="7" t="s">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B46" s="7" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A48" s="7" t="s">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B48" s="7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A49" s="8" t="s">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B49" s="8" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A50" s="8" t="s">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B50" s="8" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A53" s="8" t="s">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B53" s="8" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A54" s="7" t="s">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B54" s="7" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A55" s="8" t="s">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B55" s="8" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A56" s="8" t="s">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B56" s="8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A57" s="8" t="s">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B57" s="8" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A58" s="8" t="s">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B58" s="8" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A59" s="7" t="s">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B59" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="62" spans="1:1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A62" s="6" t="s">
+    <row r="62" spans="2:2" ht="18" x14ac:dyDescent="0.2">
+      <c r="B62" s="6" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="63" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A63" s="9" t="s">
+    <row r="63" spans="2:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="B63" s="9" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A64" s="7" t="s">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B64" s="7" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A65" s="7" t="s">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B65" s="7" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A66" s="7" t="s">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B66" s="7" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="68" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A68" s="9" t="s">
+    <row r="68" spans="2:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="B68" s="9" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A69" s="7" t="s">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B69" s="7" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A70" s="7" t="s">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B70" s="7" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A71" s="7" t="s">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B71" s="7" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A72" s="7" t="s">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B72" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A73" s="7" t="s">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B73" s="7" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A74" s="7" t="s">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B74" s="7" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="76" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A76" s="9" t="s">
+    <row r="76" spans="2:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="B76" s="9" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A77" s="7" t="s">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B77" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A78" s="7" t="s">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B78" s="7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A79" s="7" t="s">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B79" s="7" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A80" s="7" t="s">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B80" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A81" s="7" t="s">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B81" s="7" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A82" s="7" t="s">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B82" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A83" s="7" t="s">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B83" s="7" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="85" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A85" s="9" t="s">
+    <row r="85" spans="2:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="B85" s="9" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A86" s="7" t="s">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B86" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A87" s="7" t="s">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B87" s="7" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A88" s="7" t="s">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B88" s="7" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="90" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A90" s="9" t="s">
+    <row r="90" spans="2:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="B90" s="9" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A91" s="7" t="s">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B91" s="7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A92" s="7" t="s">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B92" s="7" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A93" s="7" t="s">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B93" s="7" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="95" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A95" s="9" t="s">
+    <row r="95" spans="2:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="B95" s="9" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A96" s="7" t="s">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B96" s="7" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A97" s="7" t="s">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B97" s="7" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A98" s="7" t="s">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B98" s="7" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A99" s="7" t="s">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B99" s="7" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="101" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A101" s="9" t="s">
+    <row r="101" spans="2:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="B101" s="9" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A102" s="7" t="s">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B102" s="7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A103" s="7" t="s">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B103" s="7" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A104" s="7" t="s">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B104" s="7" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="107" spans="1:1" ht="23" x14ac:dyDescent="0.25">
-      <c r="A107" s="10" t="s">
+    <row r="107" spans="2:2" ht="23" x14ac:dyDescent="0.25">
+      <c r="B107" s="10" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A108" s="8" t="s">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B108" s="8" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A109" s="8" t="s">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B109" s="8" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A110" s="8" t="s">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B110" s="8" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A111" s="8" t="s">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B111" s="8" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A112" s="8" t="s">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B112" s="8" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A113" s="8" t="s">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B113" s="8" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.15">
-      <c r="A117" s="8" t="s">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.15">
+      <c r="B117" s="8" t="s">
         <v>138</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>